<commit_message>
changes after Referesh+TMTT0037504 partial changes
</commit_message>
<xml_diff>
--- a/TestData/TMTI0068990_VerifyUserCanSearchProjectWithNameOnTimeRecordManager.xlsx
+++ b/TestData/TMTI0068990_VerifyUserCanSearchProjectWithNameOnTimeRecordManager.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vijay.kumar\source\repos\SalesForce_Project\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5AD236-85CE-4BF1-BFE5-DB481DCD27DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B943DF1-E91B-4A1D-B23B-E70ED0510D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
   <si>
     <t>Global Search User</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>120781</t>
+  </si>
+  <si>
+    <t>Omnicell, Inc.</t>
   </si>
 </sst>
 </file>
@@ -470,18 +473,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -495,22 +498,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00E5A07C-950F-4461-89EE-53C28AB50916}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -518,17 +521,20 @@
       <c r="D2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -541,16 +547,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -567,7 +573,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -584,7 +590,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -601,7 +607,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -618,7 +624,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -644,13 +650,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -661,7 +667,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
@@ -672,7 +678,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -683,7 +689,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
@@ -694,7 +700,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>

</xml_diff>